<commit_message>
Adds BAU ITC input file; integrates ITC structure into cash flows
</commit_message>
<xml_diff>
--- a/InputData/indst/BCHSR/BAU Clean Heat Subsidy Rate.xlsx
+++ b/InputData/indst/BCHSR/BAU Clean Heat Subsidy Rate.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\indst\BCHSR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\BCHSR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B695CC-A7C3-49C0-917B-4DEA43867A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14FC69B-E202-4685-A999-C3A5912AB225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2715" yWindow="2340" windowWidth="21600" windowHeight="11175" activeTab="1" xr2:uid="{9AA6BDF2-7B91-4567-88A2-0D83F9E3E450}"/>
+    <workbookView xWindow="5445" yWindow="4305" windowWidth="21600" windowHeight="12645" xr2:uid="{9AA6BDF2-7B91-4567-88A2-0D83F9E3E450}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="BCHSR" sheetId="3" r:id="rId2"/>
+    <sheet name="BCHSR-production" sheetId="3" r:id="rId2"/>
+    <sheet name="BCHSR-investment" sheetId="4" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName name="CH4_to_CO2e">'[1]Cross-Page Data'!$C$12</definedName>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>Sources:</t>
   </si>
@@ -74,10 +75,25 @@
     <t>Unit: $/BTU</t>
   </si>
   <si>
-    <t>BCHPR BAU Clean Heat Subsidy Rate</t>
+    <t>BCHPR BAU Clean Heat Investment Subsidy Rate</t>
   </si>
   <si>
-    <t>None needed. There is no Clean Heat Subsidy in the U.S. BAU.</t>
+    <t>BCHPR BAU Clean Heat Production Subsidy Rate</t>
+  </si>
+  <si>
+    <t>None needed. There are no federal clean industrial heat subsidies in the U.S.</t>
+  </si>
+  <si>
+    <t>capital costs covered by the government. Values should range between 0 and 100% (0.0-1.0).</t>
+  </si>
+  <si>
+    <t>The investment subsidy should be dimensionless, as it represents the share of</t>
+  </si>
+  <si>
+    <t>The production subsidy should be in units of 2012 USD / BTU. Values should range</t>
+  </si>
+  <si>
+    <t>up to or around approximately 1e-5 $/BTU ($10/MMBtu).</t>
   </si>
 </sst>
 </file>
@@ -136,13 +152,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -658,30 +675,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE5FEEC-01CE-4291-999E-35B30A1256CF}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1180,4 +1220,496 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE90811-281D-4C9E-85A2-D4B4CBA8A3AD}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:AE5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.28515625" customWidth="1"/>
+    <col min="2" max="3" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="3">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="3">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="3">
+        <v>2023</v>
+      </c>
+      <c r="E1" s="3">
+        <v>2024</v>
+      </c>
+      <c r="F1" s="3">
+        <v>2025</v>
+      </c>
+      <c r="G1" s="3">
+        <v>2026</v>
+      </c>
+      <c r="H1" s="3">
+        <v>2027</v>
+      </c>
+      <c r="I1" s="3">
+        <v>2028</v>
+      </c>
+      <c r="J1" s="3">
+        <v>2029</v>
+      </c>
+      <c r="K1" s="3">
+        <v>2030</v>
+      </c>
+      <c r="L1" s="3">
+        <v>2031</v>
+      </c>
+      <c r="M1" s="3">
+        <v>2032</v>
+      </c>
+      <c r="N1" s="3">
+        <v>2033</v>
+      </c>
+      <c r="O1" s="3">
+        <v>2034</v>
+      </c>
+      <c r="P1" s="3">
+        <v>2035</v>
+      </c>
+      <c r="Q1" s="3">
+        <v>2036</v>
+      </c>
+      <c r="R1" s="3">
+        <v>2037</v>
+      </c>
+      <c r="S1" s="3">
+        <v>2038</v>
+      </c>
+      <c r="T1" s="3">
+        <v>2039</v>
+      </c>
+      <c r="U1" s="3">
+        <v>2040</v>
+      </c>
+      <c r="V1" s="3">
+        <v>2041</v>
+      </c>
+      <c r="W1" s="3">
+        <v>2042</v>
+      </c>
+      <c r="X1" s="3">
+        <v>2043</v>
+      </c>
+      <c r="Y1" s="3">
+        <v>2044</v>
+      </c>
+      <c r="Z1" s="3">
+        <v>2045</v>
+      </c>
+      <c r="AA1" s="3">
+        <v>2046</v>
+      </c>
+      <c r="AB1" s="3">
+        <v>2047</v>
+      </c>
+      <c r="AC1" s="3">
+        <v>2048</v>
+      </c>
+      <c r="AD1" s="3">
+        <v>2049</v>
+      </c>
+      <c r="AE1" s="3">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>